<commit_message>
Build is now ready for research study
</commit_message>
<xml_diff>
--- a/Documents/Dissertation Readings.xlsx
+++ b/Documents/Dissertation Readings.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Pri\Documents\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\CompArchVR\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77044DF4-37C9-404C-8442-D860FC5934B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{333A7BC7-D215-4D36-A304-782E6F7EB565}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="2" xr2:uid="{23769A02-F8E7-4B96-89C2-1FAAFC8F8E1E}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{23769A02-F8E7-4B96-89C2-1FAAFC8F8E1E}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="3" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="130" uniqueCount="113">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="115">
   <si>
     <t xml:space="preserve">Database Model Visualization in Virtual Reality: A WebVR and Benediktine Space Approach </t>
   </si>
@@ -358,18 +358,6 @@
     <t>Research Period End</t>
   </si>
   <si>
-    <t>Sum</t>
-  </si>
-  <si>
-    <t>Average</t>
-  </si>
-  <si>
-    <t>Running Total</t>
-  </si>
-  <si>
-    <t>Count</t>
-  </si>
-  <si>
     <t>Start Offset</t>
   </si>
   <si>
@@ -380,6 +368,24 @@
   </si>
   <si>
     <t>Research</t>
+  </si>
+  <si>
+    <t>VR environment of digital design laboratory: a usability study</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Alnuaimi MA and Awad M </t>
+  </si>
+  <si>
+    <t>Open Link</t>
+  </si>
+  <si>
+    <t>https://doi.org/10.1016/j.cexr.2026.100159</t>
+  </si>
+  <si>
+    <t>Azin S. Janani et al</t>
+  </si>
+  <si>
+    <t>Virtual reality applications in computer science education: scoping review</t>
   </si>
 </sst>
 </file>
@@ -387,9 +393,9 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="165" formatCode="[$-14009]dd\-mm\-yyyy;@"/>
+    <numFmt numFmtId="164" formatCode="[$-14009]dd\-mm\-yyyy;@"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -411,8 +417,14 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -437,6 +449,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -451,7 +469,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1"/>
@@ -461,7 +479,8 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="1" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="1" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1042,6 +1061,7 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -1049,7 +1069,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -2035,7 +2054,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{03BFCD6E-D3AB-4E2F-B7A5-C90489B4F4C1}">
-  <dimension ref="A1:D24"/>
+  <dimension ref="A1:D27"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="100.6640625" bestFit="1" customWidth="1"/>
@@ -2314,9 +2333,41 @@
         <v>Open Link</v>
       </c>
     </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A26" t="s">
+        <v>109</v>
+      </c>
+      <c r="B26" t="s">
+        <v>110</v>
+      </c>
+      <c r="C26" s="10">
+        <v>2025</v>
+      </c>
+      <c r="D26" s="2" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A27" t="s">
+        <v>114</v>
+      </c>
+      <c r="B27" t="s">
+        <v>113</v>
+      </c>
+      <c r="C27">
+        <v>2026</v>
+      </c>
+      <c r="D27" s="2" t="s">
+        <v>112</v>
+      </c>
+    </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="D26" r:id="rId1" xr:uid="{0219E58E-C02C-4DD0-AD8C-BEE92AB76F6C}"/>
+    <hyperlink ref="D27" r:id="rId2" xr:uid="{709F2790-1040-4A8E-8EA3-F821BA08C574}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
+  <pageSetup orientation="portrait" r:id="rId3"/>
 </worksheet>
 </file>
 
@@ -2575,7 +2626,7 @@
         <v>95</v>
       </c>
       <c r="D3" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
@@ -2604,7 +2655,7 @@
         <v>42</v>
       </c>
       <c r="D5">
-        <f t="shared" ref="D5:D21" si="0">B5 - MIN($B$4:$B$18)</f>
+        <f t="shared" ref="D5:D18" si="0">B5 - MIN($B$4:$B$18)</f>
         <v>12</v>
       </c>
     </row>
@@ -2805,7 +2856,7 @@
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="B19" s="9">
         <f>B37</f>
@@ -2821,7 +2872,7 @@
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="B20" s="9">
         <f>B39</f>
@@ -2837,7 +2888,7 @@
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="B21" s="9">
         <f>B41</f>

</xml_diff>